<commit_message>
SVO Match Engine RC1 - MATCH 264 REVIEW 2
</commit_message>
<xml_diff>
--- a/ARRIVAL.xlsx
+++ b/ARRIVAL.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\SVO\Склад\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\SVO\AI\SVO_MATCH_ENGINE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{147173FD-507D-42C4-AD0B-DFB5509BA190}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE547D57-EE1F-4A00-B3C8-FECCBB0E70B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -254,16 +254,6 @@
         <rFont val="Microsoft Sans Serif"/>
         <family val="2"/>
       </rPr>
-      <t>Кондиционер для стирки, SVO парфюмированный Таинственный лотос LOTOS</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="3.5"/>
-        <rFont val="Microsoft Sans Serif"/>
-        <family val="2"/>
-      </rPr>
       <t>Кондиционер для стирки, SVO парфюмированный Цветочный туман FLORIAL 2,7</t>
     </r>
   </si>
@@ -3828,6 +3818,20 @@
         <family val="2"/>
       </rPr>
       <t>3 751 891₽</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Кондиционер для стирки, SVO парфюмированный Таинственный лотос LOTOS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="3.5"/>
+        <rFont val="Microsoft Sans Serif"/>
+        <family val="2"/>
+        <charset val="204"/>
+      </rPr>
+      <t xml:space="preserve"> 2,7 л</t>
     </r>
   </si>
 </sst>
@@ -4017,7 +4021,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -4056,6 +4060,9 @@
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" indent="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4415,7 +4422,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -4450,7 +4457,7 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="14"/>
+      <c r="A2" s="15"/>
       <c r="B2" s="2">
         <v>45410</v>
       </c>
@@ -4788,8 +4795,8 @@
       <c r="K19" s="4"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A20" s="3" t="s">
-        <v>22</v>
+      <c r="A20" s="13" t="s">
+        <v>277</v>
       </c>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -4808,7 +4815,7 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -4829,7 +4836,7 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -4850,7 +4857,7 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -4869,7 +4876,7 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -4884,7 +4891,7 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -4901,7 +4908,7 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -4918,7 +4925,7 @@
     </row>
     <row r="27" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -4937,7 +4944,7 @@
     </row>
     <row r="28" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -4952,7 +4959,7 @@
     </row>
     <row r="29" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -4967,7 +4974,7 @@
     </row>
     <row r="30" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -4986,7 +4993,7 @@
     </row>
     <row r="31" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -5007,7 +5014,7 @@
     </row>
     <row r="32" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -5024,7 +5031,7 @@
     </row>
     <row r="33" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -5039,7 +5046,7 @@
     </row>
     <row r="34" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -5054,7 +5061,7 @@
     </row>
     <row r="35" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -5071,7 +5078,7 @@
     </row>
     <row r="36" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -5086,7 +5093,7 @@
     </row>
     <row r="37" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -5105,7 +5112,7 @@
     </row>
     <row r="38" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
@@ -5120,7 +5127,7 @@
     </row>
     <row r="39" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
@@ -5139,7 +5146,7 @@
     </row>
     <row r="40" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
@@ -5158,7 +5165,7 @@
     </row>
     <row r="41" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
@@ -5177,7 +5184,7 @@
     </row>
     <row r="42" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
@@ -5194,7 +5201,7 @@
     </row>
     <row r="43" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -5209,7 +5216,7 @@
     </row>
     <row r="44" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -5226,7 +5233,7 @@
     </row>
     <row r="45" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -5241,7 +5248,7 @@
     </row>
     <row r="46" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -5260,7 +5267,7 @@
     </row>
     <row r="47" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
@@ -5277,7 +5284,7 @@
     </row>
     <row r="48" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
@@ -5294,7 +5301,7 @@
     </row>
     <row r="49" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B49" s="4"/>
       <c r="C49" s="4"/>
@@ -5311,7 +5318,7 @@
     </row>
     <row r="50" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B50" s="4"/>
       <c r="C50" s="4"/>
@@ -5328,7 +5335,7 @@
     </row>
     <row r="51" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B51" s="4"/>
       <c r="C51" s="4"/>
@@ -5347,7 +5354,7 @@
     </row>
     <row r="52" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
@@ -5366,7 +5373,7 @@
     </row>
     <row r="53" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
@@ -5385,7 +5392,7 @@
     </row>
     <row r="54" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B54" s="4"/>
       <c r="C54" s="4"/>
@@ -5402,7 +5409,7 @@
     </row>
     <row r="55" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B55" s="4"/>
       <c r="C55" s="4"/>
@@ -5423,7 +5430,7 @@
     </row>
     <row r="56" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B56" s="4"/>
       <c r="C56" s="4"/>
@@ -5442,7 +5449,7 @@
     </row>
     <row r="57" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B57" s="4"/>
       <c r="C57" s="4"/>
@@ -5459,7 +5466,7 @@
     </row>
     <row r="58" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B58" s="4"/>
       <c r="C58" s="4"/>
@@ -5480,7 +5487,7 @@
     </row>
     <row r="59" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B59" s="4"/>
       <c r="C59" s="4"/>
@@ -5501,7 +5508,7 @@
     </row>
     <row r="60" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B60" s="4"/>
       <c r="C60" s="4"/>
@@ -5518,7 +5525,7 @@
     </row>
     <row r="61" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B61" s="4"/>
       <c r="C61" s="4"/>
@@ -5535,7 +5542,7 @@
     </row>
     <row r="62" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B62" s="4"/>
       <c r="C62" s="4"/>
@@ -5552,7 +5559,7 @@
     </row>
     <row r="63" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B63" s="4"/>
       <c r="C63" s="4"/>
@@ -5569,7 +5576,7 @@
     </row>
     <row r="64" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B64" s="4"/>
       <c r="C64" s="4"/>
@@ -5584,7 +5591,7 @@
     </row>
     <row r="65" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B65" s="4"/>
       <c r="C65" s="4"/>
@@ -5601,7 +5608,7 @@
     </row>
     <row r="66" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B66" s="4"/>
       <c r="C66" s="4"/>
@@ -5616,7 +5623,7 @@
     </row>
     <row r="67" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B67" s="4"/>
       <c r="C67" s="4"/>
@@ -5633,7 +5640,7 @@
     </row>
     <row r="68" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B68" s="4"/>
       <c r="C68" s="4"/>
@@ -5648,7 +5655,7 @@
     </row>
     <row r="69" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B69" s="4"/>
       <c r="C69" s="4"/>
@@ -5663,7 +5670,7 @@
     </row>
     <row r="70" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B70" s="4"/>
       <c r="C70" s="4"/>
@@ -5678,7 +5685,7 @@
     </row>
     <row r="71" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B71" s="4"/>
       <c r="C71" s="4"/>
@@ -5695,7 +5702,7 @@
     </row>
     <row r="72" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B72" s="4"/>
       <c r="C72" s="4"/>
@@ -5712,7 +5719,7 @@
     </row>
     <row r="73" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B73" s="4"/>
       <c r="C73" s="4"/>
@@ -5729,7 +5736,7 @@
     </row>
     <row r="74" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B74" s="4"/>
       <c r="C74" s="4"/>
@@ -5746,7 +5753,7 @@
     </row>
     <row r="75" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B75" s="4"/>
       <c r="C75" s="4"/>
@@ -5763,7 +5770,7 @@
     </row>
     <row r="76" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B76" s="4"/>
       <c r="C76" s="4"/>
@@ -5780,7 +5787,7 @@
     </row>
     <row r="77" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B77" s="4"/>
       <c r="C77" s="4"/>
@@ -5797,7 +5804,7 @@
     </row>
     <row r="78" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B78" s="4"/>
       <c r="C78" s="4"/>
@@ -5814,7 +5821,7 @@
     </row>
     <row r="79" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B79" s="4"/>
       <c r="C79" s="4"/>
@@ -5831,7 +5838,7 @@
     </row>
     <row r="80" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B80" s="4"/>
       <c r="C80" s="4"/>
@@ -5848,7 +5855,7 @@
     </row>
     <row r="81" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B81" s="4"/>
       <c r="C81" s="4"/>
@@ -5865,7 +5872,7 @@
     </row>
     <row r="82" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B82" s="4"/>
       <c r="C82" s="4"/>
@@ -5882,7 +5889,7 @@
     </row>
     <row r="83" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B83" s="4"/>
       <c r="C83" s="4"/>
@@ -5897,7 +5904,7 @@
     </row>
     <row r="84" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B84" s="4"/>
       <c r="C84" s="4"/>
@@ -5912,7 +5919,7 @@
     </row>
     <row r="85" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B85" s="4"/>
       <c r="C85" s="4"/>
@@ -5929,7 +5936,7 @@
     </row>
     <row r="86" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B86" s="4"/>
       <c r="C86" s="4"/>
@@ -5944,7 +5951,7 @@
     </row>
     <row r="87" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B87" s="4"/>
       <c r="C87" s="4"/>
@@ -5959,7 +5966,7 @@
     </row>
     <row r="88" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B88" s="4"/>
       <c r="C88" s="4"/>
@@ -5976,7 +5983,7 @@
     </row>
     <row r="89" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B89" s="4"/>
       <c r="C89" s="4"/>
@@ -5993,7 +6000,7 @@
     </row>
     <row r="90" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B90" s="4"/>
       <c r="C90" s="4"/>
@@ -6010,7 +6017,7 @@
     </row>
     <row r="91" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B91" s="4"/>
       <c r="C91" s="4"/>
@@ -6027,7 +6034,7 @@
     </row>
     <row r="92" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B92" s="4"/>
       <c r="C92" s="4"/>
@@ -6044,7 +6051,7 @@
     </row>
     <row r="93" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B93" s="4"/>
       <c r="C93" s="4"/>
@@ -6061,7 +6068,7 @@
     </row>
     <row r="94" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B94" s="5">
         <v>2592</v>
@@ -6082,7 +6089,7 @@
     </row>
     <row r="95" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B95" s="5">
         <v>2592</v>
@@ -6103,7 +6110,7 @@
     </row>
     <row r="96" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B96" s="4"/>
       <c r="C96" s="4"/>
@@ -6120,7 +6127,7 @@
     </row>
     <row r="97" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B97" s="4"/>
       <c r="C97" s="4"/>
@@ -6137,7 +6144,7 @@
     </row>
     <row r="98" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B98" s="4"/>
       <c r="C98" s="4"/>
@@ -6154,7 +6161,7 @@
     </row>
     <row r="99" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B99" s="4"/>
       <c r="C99" s="4"/>
@@ -6171,7 +6178,7 @@
     </row>
     <row r="100" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B100" s="4"/>
       <c r="C100" s="4"/>
@@ -6186,7 +6193,7 @@
     </row>
     <row r="101" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B101" s="4"/>
       <c r="C101" s="4"/>
@@ -6203,7 +6210,7 @@
     </row>
     <row r="102" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B102" s="4"/>
       <c r="C102" s="4"/>
@@ -6218,7 +6225,7 @@
     </row>
     <row r="103" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B103" s="4"/>
       <c r="C103" s="4"/>
@@ -6235,7 +6242,7 @@
     </row>
     <row r="104" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B104" s="5">
         <v>312</v>
@@ -6254,7 +6261,7 @@
     </row>
     <row r="105" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B105" s="5">
         <v>312</v>
@@ -6273,7 +6280,7 @@
     </row>
     <row r="106" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B106" s="5">
         <v>312</v>
@@ -6292,7 +6299,7 @@
     </row>
     <row r="107" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B107" s="5">
         <v>312</v>
@@ -6309,7 +6316,7 @@
     </row>
     <row r="108" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B108" s="5">
         <v>312</v>
@@ -6326,7 +6333,7 @@
     </row>
     <row r="109" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B109" s="5">
         <v>312</v>
@@ -6345,7 +6352,7 @@
     </row>
     <row r="110" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B110" s="5">
         <v>312</v>
@@ -6362,7 +6369,7 @@
     </row>
     <row r="111" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B111" s="5">
         <v>312</v>
@@ -6381,7 +6388,7 @@
     </row>
     <row r="112" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B112" s="4"/>
       <c r="C112" s="4"/>
@@ -6400,7 +6407,7 @@
     </row>
     <row r="113" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B113" s="4"/>
       <c r="C113" s="4"/>
@@ -6421,7 +6428,7 @@
     </row>
     <row r="114" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B114" s="4"/>
       <c r="C114" s="4"/>
@@ -6440,7 +6447,7 @@
     </row>
     <row r="115" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B115" s="4"/>
       <c r="C115" s="4"/>
@@ -6459,7 +6466,7 @@
     </row>
     <row r="116" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B116" s="4"/>
       <c r="C116" s="4"/>
@@ -6478,7 +6485,7 @@
     </row>
     <row r="117" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B117" s="4"/>
       <c r="C117" s="4"/>
@@ -6495,7 +6502,7 @@
     </row>
     <row r="118" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B118" s="4"/>
       <c r="C118" s="4"/>
@@ -6512,7 +6519,7 @@
     </row>
     <row r="119" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B119" s="4"/>
       <c r="C119" s="4"/>
@@ -6527,7 +6534,7 @@
     </row>
     <row r="120" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B120" s="4"/>
       <c r="C120" s="4"/>
@@ -6546,7 +6553,7 @@
     </row>
     <row r="121" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B121" s="5">
         <v>168</v>
@@ -6565,7 +6572,7 @@
     </row>
     <row r="122" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B122" s="5">
         <v>162</v>
@@ -6584,7 +6591,7 @@
     </row>
     <row r="123" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B123" s="5">
         <v>156</v>
@@ -6603,7 +6610,7 @@
     </row>
     <row r="124" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B124" s="5">
         <v>168</v>
@@ -6620,7 +6627,7 @@
     </row>
     <row r="125" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B125" s="5">
         <v>180</v>
@@ -6637,7 +6644,7 @@
     </row>
     <row r="126" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B126" s="5">
         <v>174</v>
@@ -6656,7 +6663,7 @@
     </row>
     <row r="127" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B127" s="5">
         <v>174</v>
@@ -6675,7 +6682,7 @@
     </row>
     <row r="128" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B128" s="5">
         <v>162</v>
@@ -6694,7 +6701,7 @@
     </row>
     <row r="129" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B129" s="4"/>
       <c r="C129" s="4"/>
@@ -6713,7 +6720,7 @@
     </row>
     <row r="130" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B130" s="4"/>
       <c r="C130" s="4"/>
@@ -6732,7 +6739,7 @@
     </row>
     <row r="131" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B131" s="4"/>
       <c r="C131" s="4"/>
@@ -6749,7 +6756,7 @@
     </row>
     <row r="132" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B132" s="4"/>
       <c r="C132" s="4"/>
@@ -6766,7 +6773,7 @@
     </row>
     <row r="133" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B133" s="4"/>
       <c r="C133" s="4"/>
@@ -6783,7 +6790,7 @@
     </row>
     <row r="134" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B134" s="4"/>
       <c r="C134" s="4"/>
@@ -6804,7 +6811,7 @@
     </row>
     <row r="135" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B135" s="4"/>
       <c r="C135" s="4"/>
@@ -6821,7 +6828,7 @@
     </row>
     <row r="136" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B136" s="5">
         <v>112</v>
@@ -6842,7 +6849,7 @@
     </row>
     <row r="137" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B137" s="5">
         <v>104</v>
@@ -6861,7 +6868,7 @@
     </row>
     <row r="138" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B138" s="5">
         <v>104</v>
@@ -6880,7 +6887,7 @@
     </row>
     <row r="139" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B139" s="5">
         <v>112</v>
@@ -6901,7 +6908,7 @@
     </row>
     <row r="140" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B140" s="5">
         <v>104</v>
@@ -6920,7 +6927,7 @@
     </row>
     <row r="141" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B141" s="5">
         <v>112</v>
@@ -6941,7 +6948,7 @@
     </row>
     <row r="142" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B142" s="5">
         <v>104</v>
@@ -6962,7 +6969,7 @@
     </row>
     <row r="143" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B143" s="4"/>
       <c r="C143" s="4"/>
@@ -6981,7 +6988,7 @@
     </row>
     <row r="144" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A144" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B144" s="4"/>
       <c r="C144" s="4"/>
@@ -7000,7 +7007,7 @@
     </row>
     <row r="145" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B145" s="4"/>
       <c r="C145" s="4"/>
@@ -7021,7 +7028,7 @@
     </row>
     <row r="146" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B146" s="4"/>
       <c r="C146" s="4"/>
@@ -7038,7 +7045,7 @@
     </row>
     <row r="147" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B147" s="5">
         <v>111</v>
@@ -7055,7 +7062,7 @@
     </row>
     <row r="148" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A148" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B148" s="5">
         <v>111</v>
@@ -7074,7 +7081,7 @@
     </row>
     <row r="149" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B149" s="5">
         <v>111</v>
@@ -7093,7 +7100,7 @@
     </row>
     <row r="150" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B150" s="5">
         <v>111</v>
@@ -7114,7 +7121,7 @@
     </row>
     <row r="151" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" s="3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B151" s="5">
         <v>111</v>
@@ -7135,7 +7142,7 @@
     </row>
     <row r="152" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B152" s="4"/>
       <c r="C152" s="4"/>
@@ -7150,7 +7157,7 @@
     </row>
     <row r="153" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B153" s="4"/>
       <c r="C153" s="4"/>
@@ -7165,7 +7172,7 @@
     </row>
     <row r="154" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B154" s="4"/>
       <c r="C154" s="4"/>
@@ -7180,7 +7187,7 @@
     </row>
     <row r="155" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A155" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B155" s="5">
         <v>111</v>
@@ -7197,7 +7204,7 @@
     </row>
     <row r="156" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B156" s="5">
         <v>74</v>
@@ -7216,7 +7223,7 @@
     </row>
     <row r="157" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B157" s="5">
         <v>74</v>
@@ -7233,7 +7240,7 @@
     </row>
     <row r="158" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A158" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B158" s="5">
         <v>74</v>
@@ -7254,7 +7261,7 @@
     </row>
     <row r="159" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A159" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B159" s="5">
         <v>74</v>
@@ -7275,7 +7282,7 @@
     </row>
     <row r="160" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A160" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B160" s="5">
         <v>74</v>
@@ -7296,7 +7303,7 @@
     </row>
     <row r="161" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A161" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B161" s="5">
         <v>74</v>
@@ -7315,7 +7322,7 @@
     </row>
     <row r="162" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A162" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B162" s="4"/>
       <c r="C162" s="4"/>
@@ -7330,7 +7337,7 @@
     </row>
     <row r="163" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A163" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B163" s="4"/>
       <c r="C163" s="4"/>
@@ -7347,7 +7354,7 @@
     </row>
     <row r="164" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A164" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B164" s="4"/>
       <c r="C164" s="4"/>
@@ -7364,7 +7371,7 @@
     </row>
     <row r="165" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A165" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B165" s="4"/>
       <c r="C165" s="4"/>
@@ -7381,7 +7388,7 @@
     </row>
     <row r="166" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A166" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B166" s="4"/>
       <c r="C166" s="4"/>
@@ -7400,7 +7407,7 @@
     </row>
     <row r="167" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A167" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B167" s="4"/>
       <c r="C167" s="4"/>
@@ -7419,7 +7426,7 @@
     </row>
     <row r="168" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A168" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B168" s="4"/>
       <c r="C168" s="4"/>
@@ -7436,7 +7443,7 @@
     </row>
     <row r="169" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A169" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B169" s="4"/>
       <c r="C169" s="4"/>
@@ -7453,7 +7460,7 @@
     </row>
     <row r="170" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A170" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B170" s="4"/>
       <c r="C170" s="4"/>
@@ -7470,7 +7477,7 @@
     </row>
     <row r="171" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A171" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B171" s="4"/>
       <c r="C171" s="4"/>
@@ -7487,7 +7494,7 @@
     </row>
     <row r="172" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A172" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B172" s="4"/>
       <c r="C172" s="4"/>
@@ -7504,7 +7511,7 @@
     </row>
     <row r="173" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A173" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B173" s="4"/>
       <c r="C173" s="4"/>
@@ -7521,7 +7528,7 @@
     </row>
     <row r="174" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A174" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B174" s="4"/>
       <c r="C174" s="4"/>
@@ -7538,7 +7545,7 @@
     </row>
     <row r="175" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A175" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B175" s="4"/>
       <c r="C175" s="4"/>
@@ -7555,7 +7562,7 @@
     </row>
     <row r="176" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A176" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B176" s="5">
         <v>7000</v>
@@ -7574,7 +7581,7 @@
     </row>
     <row r="177" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A177" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B177" s="4"/>
       <c r="C177" s="5">
@@ -7601,7 +7608,7 @@
     </row>
     <row r="178" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A178" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B178" s="4"/>
       <c r="C178" s="5">
@@ -7624,7 +7631,7 @@
     </row>
     <row r="179" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A179" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B179" s="4"/>
       <c r="C179" s="5">
@@ -7649,7 +7656,7 @@
     </row>
     <row r="180" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A180" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B180" s="4"/>
       <c r="C180" s="5">
@@ -7676,7 +7683,7 @@
     </row>
     <row r="181" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A181" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B181" s="4"/>
       <c r="C181" s="5">
@@ -7701,7 +7708,7 @@
     </row>
     <row r="182" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A182" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B182" s="4"/>
       <c r="C182" s="4"/>
@@ -7720,7 +7727,7 @@
     </row>
     <row r="183" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A183" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B183" s="4"/>
       <c r="C183" s="5">
@@ -7745,7 +7752,7 @@
     </row>
     <row r="184" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A184" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B184" s="4"/>
       <c r="C184" s="4"/>
@@ -7764,7 +7771,7 @@
     </row>
     <row r="185" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A185" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B185" s="4"/>
       <c r="C185" s="5">
@@ -7791,7 +7798,7 @@
     </row>
     <row r="186" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A186" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B186" s="4"/>
       <c r="C186" s="4"/>
@@ -7808,7 +7815,7 @@
     </row>
     <row r="187" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A187" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B187" s="4"/>
       <c r="C187" s="5">
@@ -7831,7 +7838,7 @@
     </row>
     <row r="188" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A188" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B188" s="4"/>
       <c r="C188" s="4"/>
@@ -7850,7 +7857,7 @@
     </row>
     <row r="189" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A189" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B189" s="4"/>
       <c r="C189" s="5">
@@ -7877,7 +7884,7 @@
     </row>
     <row r="190" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A190" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B190" s="4"/>
       <c r="C190" s="5">
@@ -7900,7 +7907,7 @@
     </row>
     <row r="191" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A191" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B191" s="4"/>
       <c r="C191" s="5">
@@ -7921,7 +7928,7 @@
     </row>
     <row r="192" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A192" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B192" s="4"/>
       <c r="C192" s="4"/>
@@ -7940,7 +7947,7 @@
     </row>
     <row r="193" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A193" s="3" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B193" s="4"/>
       <c r="C193" s="5">
@@ -7965,7 +7972,7 @@
     </row>
     <row r="194" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A194" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B194" s="4"/>
       <c r="C194" s="5">
@@ -7988,7 +7995,7 @@
     </row>
     <row r="195" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A195" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B195" s="4"/>
       <c r="C195" s="5">
@@ -8011,7 +8018,7 @@
     </row>
     <row r="196" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A196" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B196" s="4"/>
       <c r="C196" s="5">
@@ -8032,7 +8039,7 @@
     </row>
     <row r="197" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A197" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B197" s="4"/>
       <c r="C197" s="4"/>
@@ -8051,7 +8058,7 @@
     </row>
     <row r="198" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A198" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B198" s="4"/>
       <c r="C198" s="5">
@@ -8070,7 +8077,7 @@
     </row>
     <row r="199" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A199" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B199" s="4"/>
       <c r="C199" s="4"/>
@@ -8091,7 +8098,7 @@
     </row>
     <row r="200" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A200" s="3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B200" s="4"/>
       <c r="C200" s="4"/>
@@ -8110,7 +8117,7 @@
     </row>
     <row r="201" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A201" s="3" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B201" s="4"/>
       <c r="C201" s="4"/>
@@ -8129,7 +8136,7 @@
     </row>
     <row r="202" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A202" s="3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B202" s="4"/>
       <c r="C202" s="4"/>
@@ -8150,7 +8157,7 @@
     </row>
     <row r="203" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A203" s="3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B203" s="4"/>
       <c r="C203" s="4"/>
@@ -8171,7 +8178,7 @@
     </row>
     <row r="204" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A204" s="3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B204" s="4"/>
       <c r="C204" s="4"/>
@@ -8190,7 +8197,7 @@
     </row>
     <row r="205" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A205" s="3" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B205" s="4"/>
       <c r="C205" s="4"/>
@@ -8209,7 +8216,7 @@
     </row>
     <row r="206" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A206" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B206" s="4"/>
       <c r="C206" s="4"/>
@@ -8232,7 +8239,7 @@
     </row>
     <row r="207" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A207" s="3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B207" s="4"/>
       <c r="C207" s="4"/>
@@ -8251,7 +8258,7 @@
     </row>
     <row r="208" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A208" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B208" s="4"/>
       <c r="C208" s="4"/>
@@ -8272,7 +8279,7 @@
     </row>
     <row r="209" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A209" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B209" s="4"/>
       <c r="C209" s="4"/>
@@ -8291,7 +8298,7 @@
     </row>
     <row r="210" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A210" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B210" s="4"/>
       <c r="C210" s="4"/>
@@ -8310,7 +8317,7 @@
     </row>
     <row r="211" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A211" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B211" s="4"/>
       <c r="C211" s="4"/>
@@ -8331,7 +8338,7 @@
     </row>
     <row r="212" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A212" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B212" s="4"/>
       <c r="C212" s="4"/>
@@ -8350,7 +8357,7 @@
     </row>
     <row r="213" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A213" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B213" s="4"/>
       <c r="C213" s="4"/>
@@ -8369,7 +8376,7 @@
     </row>
     <row r="214" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A214" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B214" s="4"/>
       <c r="C214" s="4"/>
@@ -8388,7 +8395,7 @@
     </row>
     <row r="215" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A215" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B215" s="4"/>
       <c r="C215" s="4"/>
@@ -8407,7 +8414,7 @@
     </row>
     <row r="216" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A216" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B216" s="4"/>
       <c r="C216" s="4"/>
@@ -8424,7 +8431,7 @@
     </row>
     <row r="217" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A217" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B217" s="4"/>
       <c r="C217" s="4"/>
@@ -8443,7 +8450,7 @@
     </row>
     <row r="218" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A218" s="3" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B218" s="4"/>
       <c r="C218" s="4"/>
@@ -8460,7 +8467,7 @@
     </row>
     <row r="219" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A219" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B219" s="4"/>
       <c r="C219" s="4"/>
@@ -8475,7 +8482,7 @@
     </row>
     <row r="220" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A220" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B220" s="4"/>
       <c r="C220" s="4"/>
@@ -8492,7 +8499,7 @@
     </row>
     <row r="221" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A221" s="3" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B221" s="4"/>
       <c r="C221" s="4"/>
@@ -8509,7 +8516,7 @@
     </row>
     <row r="222" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A222" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B222" s="4"/>
       <c r="C222" s="4"/>
@@ -8526,7 +8533,7 @@
     </row>
     <row r="223" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A223" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B223" s="4"/>
       <c r="C223" s="4"/>
@@ -8543,7 +8550,7 @@
     </row>
     <row r="224" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A224" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B224" s="4"/>
       <c r="C224" s="4"/>
@@ -8560,7 +8567,7 @@
     </row>
     <row r="225" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A225" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B225" s="4"/>
       <c r="C225" s="4"/>
@@ -8577,7 +8584,7 @@
     </row>
     <row r="226" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A226" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B226" s="4"/>
       <c r="C226" s="4"/>
@@ -8594,7 +8601,7 @@
     </row>
     <row r="227" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A227" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B227" s="4"/>
       <c r="C227" s="4"/>
@@ -8611,7 +8618,7 @@
     </row>
     <row r="228" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A228" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B228" s="4"/>
       <c r="C228" s="4"/>
@@ -8628,7 +8635,7 @@
     </row>
     <row r="229" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A229" s="3" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B229" s="4"/>
       <c r="C229" s="4"/>
@@ -8645,7 +8652,7 @@
     </row>
     <row r="230" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A230" s="3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B230" s="4"/>
       <c r="C230" s="4"/>
@@ -8662,7 +8669,7 @@
     </row>
     <row r="231" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A231" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B231" s="4"/>
       <c r="C231" s="4"/>
@@ -8679,7 +8686,7 @@
     </row>
     <row r="232" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A232" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B232" s="4"/>
       <c r="C232" s="4"/>
@@ -8696,7 +8703,7 @@
     </row>
     <row r="233" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A233" s="3" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B233" s="4"/>
       <c r="C233" s="4"/>
@@ -8713,7 +8720,7 @@
     </row>
     <row r="234" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A234" s="3" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B234" s="4"/>
       <c r="C234" s="4"/>
@@ -8734,7 +8741,7 @@
     </row>
     <row r="235" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A235" s="3" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B235" s="4"/>
       <c r="C235" s="4"/>
@@ -8755,7 +8762,7 @@
     </row>
     <row r="236" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A236" s="3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B236" s="4"/>
       <c r="C236" s="4"/>
@@ -8776,7 +8783,7 @@
     </row>
     <row r="237" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A237" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B237" s="4"/>
       <c r="C237" s="4"/>
@@ -8795,7 +8802,7 @@
     </row>
     <row r="238" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A238" s="3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B238" s="4"/>
       <c r="C238" s="4"/>
@@ -8814,7 +8821,7 @@
     </row>
     <row r="239" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A239" s="3" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B239" s="4"/>
       <c r="C239" s="4"/>
@@ -8833,7 +8840,7 @@
     </row>
     <row r="240" spans="1:11" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A240" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B240" s="4"/>
       <c r="C240" s="4"/>
@@ -8850,7 +8857,7 @@
     </row>
     <row r="241" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A241" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B241" s="4"/>
       <c r="C241" s="4"/>
@@ -8867,7 +8874,7 @@
     </row>
     <row r="242" spans="1:11" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A242" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B242" s="4"/>
       <c r="C242" s="4"/>
@@ -8884,7 +8891,7 @@
     </row>
     <row r="243" spans="1:11" ht="8.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A243" s="9" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B243" s="4"/>
       <c r="C243" s="4"/>
@@ -8901,7 +8908,7 @@
     </row>
     <row r="244" spans="1:11" ht="8.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A244" s="9" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B244" s="4"/>
       <c r="C244" s="4"/>
@@ -8918,7 +8925,7 @@
     </row>
     <row r="245" spans="1:11" ht="8.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A245" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B245" s="4"/>
       <c r="C245" s="4"/>
@@ -8935,7 +8942,7 @@
     </row>
     <row r="246" spans="1:11" ht="8.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A246" s="9" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B246" s="4"/>
       <c r="C246" s="4"/>
@@ -8952,7 +8959,7 @@
     </row>
     <row r="247" spans="1:11" ht="8.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A247" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B247" s="4"/>
       <c r="C247" s="4"/>
@@ -8969,7 +8976,7 @@
     </row>
     <row r="248" spans="1:11" ht="8.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A248" s="9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B248" s="4"/>
       <c r="C248" s="4"/>
@@ -8986,7 +8993,7 @@
     </row>
     <row r="249" spans="1:11" ht="8.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A249" s="9" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B249" s="4"/>
       <c r="C249" s="4"/>
@@ -9003,7 +9010,7 @@
     </row>
     <row r="250" spans="1:11" ht="8.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A250" s="9" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B250" s="4"/>
       <c r="C250" s="4"/>
@@ -9020,7 +9027,7 @@
     </row>
     <row r="251" spans="1:11" ht="8.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A251" s="9" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B251" s="4"/>
       <c r="C251" s="4"/>
@@ -9037,7 +9044,7 @@
     </row>
     <row r="252" spans="1:11" ht="8.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A252" s="9" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B252" s="4"/>
       <c r="C252" s="4"/>
@@ -9054,7 +9061,7 @@
     </row>
     <row r="253" spans="1:11" ht="8.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A253" s="9" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B253" s="4"/>
       <c r="C253" s="5">
@@ -9073,7 +9080,7 @@
     </row>
     <row r="254" spans="1:11" ht="8.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A254" s="9" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B254" s="4"/>
       <c r="C254" s="5">
@@ -9092,7 +9099,7 @@
     </row>
     <row r="255" spans="1:11" ht="8.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A255" s="9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B255" s="4"/>
       <c r="C255" s="5">
@@ -9111,7 +9118,7 @@
     </row>
     <row r="256" spans="1:11" ht="8.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A256" s="9" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B256" s="4"/>
       <c r="C256" s="5">
@@ -9130,7 +9137,7 @@
     </row>
     <row r="257" spans="1:11" ht="8.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A257" s="9" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B257" s="4"/>
       <c r="C257" s="4"/>
@@ -9147,7 +9154,7 @@
     </row>
     <row r="258" spans="1:11" ht="8.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A258" s="9" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B258" s="4"/>
       <c r="C258" s="4"/>
@@ -9164,7 +9171,7 @@
     </row>
     <row r="259" spans="1:11" ht="8.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A259" s="9" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B259" s="4"/>
       <c r="C259" s="4"/>
@@ -9181,7 +9188,7 @@
     </row>
     <row r="260" spans="1:11" ht="8.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A260" s="9" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B260" s="4"/>
       <c r="C260" s="5">
@@ -9200,7 +9207,7 @@
     </row>
     <row r="261" spans="1:11" ht="8.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A261" s="9" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B261" s="4"/>
       <c r="C261" s="4"/>
@@ -9217,7 +9224,7 @@
     </row>
     <row r="262" spans="1:11" ht="8.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A262" s="9" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B262" s="4"/>
       <c r="C262" s="4"/>
@@ -9234,7 +9241,7 @@
     </row>
     <row r="263" spans="1:11" ht="8.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A263" s="9" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B263" s="4"/>
       <c r="C263" s="4"/>
@@ -9253,7 +9260,7 @@
     </row>
     <row r="264" spans="1:11" ht="8.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A264" s="9" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B264" s="4"/>
       <c r="C264" s="4"/>
@@ -9270,7 +9277,7 @@
     </row>
     <row r="265" spans="1:11" ht="8.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A265" s="9" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B265" s="4"/>
       <c r="C265" s="4"/>
@@ -9287,7 +9294,7 @@
     </row>
     <row r="266" spans="1:11" ht="8.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A266" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B266" s="4"/>
       <c r="C266" s="4"/>
@@ -9304,7 +9311,7 @@
     </row>
     <row r="267" spans="1:11" ht="8.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A267" s="9" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B267" s="4"/>
       <c r="C267" s="4"/>
@@ -9323,7 +9330,7 @@
     </row>
     <row r="268" spans="1:11" ht="8.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A268" s="9" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B268" s="4"/>
       <c r="C268" s="4"/>
@@ -9343,28 +9350,28 @@
     <row r="269" spans="1:11" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A269" s="4"/>
       <c r="B269" s="10" t="s">
+        <v>270</v>
+      </c>
+      <c r="C269" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="C269" s="1" t="s">
+      <c r="D269" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="D269" s="1" t="s">
+      <c r="E269" s="1" t="s">
         <v>273</v>
-      </c>
-      <c r="E269" s="1" t="s">
-        <v>274</v>
       </c>
       <c r="F269" s="11">
         <v>20091721</v>
       </c>
       <c r="G269" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="H269" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="H269" s="1" t="s">
+      <c r="I269" s="1" t="s">
         <v>276</v>
-      </c>
-      <c r="I269" s="1" t="s">
-        <v>277</v>
       </c>
       <c r="J269" s="11">
         <v>1481964</v>

</xml_diff>